<commit_message>
Merge Module/Task cells and add Status column
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01319BznfEv5w8UGSo5VivdJ
</commit_message>
<xml_diff>
--- a/docs/KONU_BRD_Functionalities.xlsx
+++ b/docs/KONU_BRD_Functionalities.xlsx
@@ -10,7 +10,7 @@
     <sheet name="KONU Functionalities" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'KONU Functionalities'!$A$1:$C$160</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'KONU Functionalities'!$A$1:$D$160</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -61,7 +61,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -74,11 +74,20 @@
         <color rgb="00BBBBBB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -88,6 +97,13 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -454,12 +470,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C160"/>
+  <dimension ref="A1:D160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,14 +495,19 @@
           <t>Sub Task</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>NFR – Platform Requirements</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>NFR-01 Availability</t>
         </is>
@@ -495,14 +517,14 @@
           <t>Monitor launch-critical flows</t>
         </is>
       </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>NFR-01 Availability</t>
         </is>
@@ -512,14 +534,14 @@
           <t>Define incident ownership</t>
         </is>
       </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>NFR-02 Performance</t>
         </is>
@@ -529,31 +551,27 @@
           <t>Set performance budgets for search/detail/map</t>
         </is>
       </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>NFR-02 Performance</t>
-        </is>
-      </c>
+      <c r="B5" s="5" t="n"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Measure in launch environment</t>
         </is>
       </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>NFR-03 Security</t>
         </is>
@@ -563,48 +581,39 @@
           <t>Authentication &amp; authorization</t>
         </is>
       </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>NFR-03 Security</t>
-        </is>
-      </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Secrets management &amp; audit logs</t>
         </is>
       </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>NFR-03 Security</t>
-        </is>
-      </c>
+      <c r="B8" s="5" t="n"/>
       <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Vulnerability remediation as release gate</t>
         </is>
       </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>NFR-04 Privacy</t>
         </is>
@@ -614,48 +623,39 @@
           <t>Consent &amp; data minimization</t>
         </is>
       </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>NFR-04 Privacy</t>
-        </is>
-      </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Role access</t>
         </is>
       </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>NFR-04 Privacy</t>
-        </is>
-      </c>
+      <c r="B11" s="5" t="n"/>
       <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Deletion/retention rules</t>
         </is>
       </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>NFR-05 Observability</t>
         </is>
@@ -665,31 +665,27 @@
           <t>Logs/metrics for critical APIs, AI calls, pipelines</t>
         </is>
       </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>NFR-05 Observability</t>
-        </is>
-      </c>
+      <c r="B13" s="5" t="n"/>
       <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Logs/metrics for payments/service requests</t>
         </is>
       </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>NFR-06 Analytics</t>
         </is>
@@ -699,14 +695,14 @@
           <t>Instrument funnel: discovery → lead/service request → fulfilment</t>
         </is>
       </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>NFR-07 Accessibility</t>
         </is>
@@ -716,48 +712,39 @@
           <t>Readable contrast</t>
         </is>
       </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>NFR-07 Accessibility</t>
-        </is>
-      </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Keyboard/focus behaviour</t>
         </is>
       </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>NFR-07 Accessibility</t>
-        </is>
-      </c>
+      <c r="B17" s="5" t="n"/>
       <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Semantic labelling</t>
         </is>
       </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>NFR-08 Scalability</t>
         </is>
@@ -767,31 +754,33 @@
           <t>Avoid single points of failure</t>
         </is>
       </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>NFR – Platform Requirements</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>NFR-08 Scalability</t>
-        </is>
-      </c>
+      <c r="A19" s="5" t="n"/>
+      <c r="B19" s="5" t="n"/>
       <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Document expected load assumptions</t>
         </is>
       </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>A – Core Listings, Search &amp; Property Detail</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>CL-01 Search &amp; filters</t>
         </is>
@@ -801,14 +790,14 @@
           <t>Filter by location, type, price, core attributes</t>
         </is>
       </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>CL-01 Search &amp; filters</t>
         </is>
@@ -818,14 +807,14 @@
           <t>Preserve selected filters</t>
         </is>
       </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>CL-02 Property card/detail</t>
         </is>
@@ -835,48 +824,39 @@
           <t>Show standardized core facts</t>
         </is>
       </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>CL-02 Property card/detail</t>
-        </is>
-      </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Show last-updated &amp; verification badge</t>
         </is>
       </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>CL-02 Property card/detail</t>
-        </is>
-      </c>
+      <c r="B24" s="5" t="n"/>
       <c r="C24" s="3" t="inlineStr">
         <is>
           <t>Never show missing data as verified</t>
         </is>
       </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>CL-03 Map/list sync</t>
         </is>
@@ -886,31 +866,27 @@
           <t>Sync selection/filter between views</t>
         </is>
       </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>CL-03 Map/list sync</t>
-        </is>
-      </c>
+      <c r="B26" s="5" t="n"/>
       <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Keep property counts consistent (except clustering)</t>
         </is>
       </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>CL-04 Save/favorite</t>
         </is>
@@ -920,48 +896,39 @@
           <t>Save property to account</t>
         </is>
       </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>CL-04 Save/favorite</t>
-        </is>
-      </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Remove saved property</t>
         </is>
       </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>CL-04 Save/favorite</t>
-        </is>
-      </c>
+      <c r="B29" s="5" t="n"/>
       <c r="C29" s="3" t="inlineStr">
         <is>
           <t>Persist after login</t>
         </is>
       </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>CL-05 Lead/service CTA</t>
         </is>
@@ -971,31 +938,27 @@
           <t>Route enquiry to CRM/ops</t>
         </is>
       </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>CL-05 Lead/service CTA</t>
-        </is>
-      </c>
+      <c r="B31" s="5" t="n"/>
       <c r="C31" s="3" t="inlineStr">
         <is>
           <t>Capture source, property/project ID, contact/consent, timestamp, campaign</t>
         </is>
       </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>CL-06 Admin listing management</t>
         </is>
@@ -1005,48 +968,39 @@
           <t>Create/update/deactivate listing</t>
         </is>
       </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>CL-06 Admin listing management</t>
-        </is>
-      </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
           <t>Audit trail by user/time</t>
         </is>
       </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>CL-06 Admin listing management</t>
-        </is>
-      </c>
+      <c r="B34" s="5" t="n"/>
       <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Hide deactivated inventory from public</t>
         </is>
       </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>CL-07 Duplicate/stale flagging</t>
         </is>
@@ -1056,31 +1010,27 @@
           <t>Flag duplicate/stale records via admin rules</t>
         </is>
       </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>CL-07 Duplicate/stale flagging</t>
-        </is>
-      </c>
+      <c r="B36" s="5" t="n"/>
       <c r="C36" s="3" t="inlineStr">
         <is>
           <t>Review without auto-deletion</t>
         </is>
       </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>CL-08 Personalized discovery</t>
         </is>
@@ -1090,31 +1040,27 @@
           <t>Use searches, views, saves, location, budget, configuration, amenities</t>
         </is>
       </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>CL-08 Personalized discovery</t>
-        </is>
-      </c>
+      <c r="B38" s="5" t="n"/>
       <c r="C38" s="3" t="inlineStr">
         <is>
           <t>Apply consent/privacy controls</t>
         </is>
       </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>CL-09 Engagement metrics</t>
         </is>
@@ -1124,48 +1070,45 @@
           <t>Capture views and saves per listing</t>
         </is>
       </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>CL-09 Engagement metrics</t>
-        </is>
-      </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
           <t>Apply agreed counting rules</t>
         </is>
       </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>A – Core Listings, Search &amp; Property Detail</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>CL-09 Engagement metrics</t>
-        </is>
-      </c>
+      <c r="A41" s="5" t="n"/>
+      <c r="B41" s="5" t="n"/>
       <c r="C41" s="3" t="inlineStr">
         <is>
           <t>Listing-level analytics</t>
         </is>
       </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>B – GIS &amp; Hyperlocal Intelligence</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>GIS-01 Geocoded location</t>
         </is>
@@ -1175,14 +1118,14 @@
           <t>Show property on base map</t>
         </is>
       </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>B – GIS &amp; Hyperlocal Intelligence</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>GIS-01 Geocoded location</t>
         </is>
@@ -1192,14 +1135,14 @@
           <t>Meet documented accuracy</t>
         </is>
       </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>B – GIS &amp; Hyperlocal Intelligence</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>GIS-02 Infrastructure/POI layers</t>
         </is>
@@ -1209,48 +1152,39 @@
           <t>ORR/RRR/metro/flyovers &amp; amenity layers</t>
         </is>
       </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>B – GIS &amp; Hyperlocal Intelligence</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>GIS-02 Infrastructure/POI layers</t>
-        </is>
-      </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
           <t>Toggle layers</t>
         </is>
       </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>B – GIS &amp; Hyperlocal Intelligence</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>GIS-02 Infrastructure/POI layers</t>
-        </is>
-      </c>
+      <c r="B46" s="5" t="n"/>
       <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Source &amp; last-updated metadata</t>
         </is>
       </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>B – GIS &amp; Hyperlocal Intelligence</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>GIS-03 Boundary overlays</t>
         </is>
@@ -1260,31 +1194,27 @@
           <t>Locality boundary overlays for launch geographies</t>
         </is>
       </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>B – GIS &amp; Hyperlocal Intelligence</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>GIS-03 Boundary overlays</t>
-        </is>
-      </c>
+      <c r="B48" s="5" t="n"/>
       <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Error-free geometry</t>
         </is>
       </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>B – GIS &amp; Hyperlocal Intelligence</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>GIS-04 Graceful API failure</t>
         </is>
@@ -1294,31 +1224,27 @@
           <t>Handle timeout/error without breaking property page</t>
         </is>
       </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>B – GIS &amp; Hyperlocal Intelligence</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>GIS-04 Graceful API failure</t>
-        </is>
-      </c>
+      <c r="B50" s="5" t="n"/>
       <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Monitor &amp; expose error data to ops</t>
         </is>
       </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>B – GIS &amp; Hyperlocal Intelligence</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>GIS-05 Spatial dataset updates</t>
         </is>
@@ -1328,48 +1254,39 @@
           <t>Controlled dataset update</t>
         </is>
       </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>B – GIS &amp; Hyperlocal Intelligence</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>GIS-05 Spatial dataset updates</t>
-        </is>
-      </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
           <t>Record version &amp; effective date</t>
         </is>
       </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>B – GIS &amp; Hyperlocal Intelligence</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>GIS-05 Spatial dataset updates</t>
-        </is>
-      </c>
+      <c r="B53" s="5" t="n"/>
       <c r="C53" s="2" t="inlineStr">
         <is>
           <t>Rollback</t>
         </is>
       </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>B – GIS &amp; Hyperlocal Intelligence</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>GIS-06 Nearby updates</t>
         </is>
@@ -1379,31 +1296,33 @@
           <t>Detect new properties/developments/infra within approved radius</t>
         </is>
       </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>B – GIS &amp; Hyperlocal Intelligence</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>GIS-06 Nearby updates</t>
-        </is>
-      </c>
+      <c r="A55" s="5" t="n"/>
+      <c r="B55" s="5" t="n"/>
       <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Show on dashboard &amp; notification channels</t>
         </is>
       </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>C – Kestimate</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B56" s="6" t="inlineStr">
         <is>
           <t>KE-01 Estimate request/view</t>
         </is>
@@ -1413,14 +1332,14 @@
           <t>Return estimate for supported types/areas</t>
         </is>
       </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>C – Kestimate</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>KE-01 Estimate request/view</t>
         </is>
@@ -1430,14 +1349,14 @@
           <t>Insufficient-data state; no fabricated values</t>
         </is>
       </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>C – Kestimate</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>KE-02 Range/confidence</t>
         </is>
@@ -1447,31 +1366,27 @@
           <t>Show range/confidence indicator</t>
         </is>
       </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>C – Kestimate</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>KE-02 Range/confidence</t>
-        </is>
-      </c>
+      <c r="B59" s="5" t="n"/>
       <c r="C59" s="3" t="inlineStr">
         <is>
           <t>No single unexplained value</t>
         </is>
       </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t>C – Kestimate</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B60" s="6" t="inlineStr">
         <is>
           <t>KE-03 Audit traceability</t>
         </is>
@@ -1481,31 +1396,27 @@
           <t>Store model version, timestamp, input features</t>
         </is>
       </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>C – Kestimate</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="inlineStr">
-        <is>
-          <t>KE-03 Audit traceability</t>
-        </is>
-      </c>
+      <c r="B61" s="5" t="n"/>
       <c r="C61" s="3" t="inlineStr">
         <is>
           <t>Apply privacy controls</t>
         </is>
       </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>C – Kestimate</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="B62" s="6" t="inlineStr">
         <is>
           <t>KE-04 Explainability</t>
         </is>
@@ -1515,14 +1426,14 @@
           <t>Show top value drivers/comparables in plain language</t>
         </is>
       </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>C – Kestimate</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="inlineStr">
+      <c r="B63" s="6" t="inlineStr">
         <is>
           <t>KE-05 Data-quality rules</t>
         </is>
@@ -1532,48 +1443,39 @@
           <t>Define thresholds for missing/stale/outlier inputs</t>
         </is>
       </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="inlineStr">
-        <is>
-          <t>C – Kestimate</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>KE-05 Data-quality rules</t>
-        </is>
-      </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
           <t>Fallback behaviour</t>
         </is>
       </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="inlineStr">
-        <is>
-          <t>C – Kestimate</t>
-        </is>
-      </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>KE-05 Data-quality rules</t>
-        </is>
-      </c>
+      <c r="B65" s="5" t="n"/>
       <c r="C65" s="3" t="inlineStr">
         <is>
           <t>Log exceptions</t>
         </is>
       </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>C – Kestimate</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B66" s="6" t="inlineStr">
         <is>
           <t>KE-06 Monitoring</t>
         </is>
@@ -1583,31 +1485,27 @@
           <t>Track errors, latency, coverage, drift/quality</t>
         </is>
       </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t>C – Kestimate</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>KE-06 Monitoring</t>
-        </is>
-      </c>
+      <c r="B67" s="5" t="n"/>
       <c r="C67" s="3" t="inlineStr">
         <is>
           <t>Segment by geography/property type</t>
         </is>
       </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="inlineStr">
-        <is>
-          <t>C – Kestimate</t>
-        </is>
-      </c>
-      <c r="B68" s="3" t="inlineStr">
+      <c r="B68" s="6" t="inlineStr">
         <is>
           <t>KE-07 Legal disclaimer</t>
         </is>
@@ -1617,14 +1515,14 @@
           <t>Show 'informational, not certified valuation' wherever displayed/shared</t>
         </is>
       </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="3" t="inlineStr">
-        <is>
-          <t>C – Kestimate</t>
-        </is>
-      </c>
-      <c r="B69" s="3" t="inlineStr">
+      <c r="B69" s="6" t="inlineStr">
         <is>
           <t>KE-08 GIS-driven refresh</t>
         </is>
@@ -1634,31 +1532,33 @@
           <t>Use infra/development/connectivity changes as inputs</t>
         </is>
       </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="3" t="inlineStr">
-        <is>
-          <t>C – Kestimate</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>KE-08 GIS-driven refresh</t>
-        </is>
-      </c>
+      <c r="A70" s="5" t="n"/>
+      <c r="B70" s="5" t="n"/>
       <c r="C70" s="3" t="inlineStr">
         <is>
           <t>Refresh current estimates &amp; future projections</t>
         </is>
       </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr">
+      <c r="A71" s="4" t="inlineStr">
         <is>
           <t>D – Bujji AI Property Assistant</t>
         </is>
       </c>
-      <c r="B71" s="2" t="inlineStr">
+      <c r="B71" s="4" t="inlineStr">
         <is>
           <t>AI-01 Grounded answers</t>
         </is>
@@ -1668,14 +1568,14 @@
           <t>Answer from approved sources &amp; user/property context</t>
         </is>
       </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>D – Bujji AI Property Assistant</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
+      <c r="B72" s="4" t="inlineStr">
         <is>
           <t>AI-01 Grounded answers</t>
         </is>
@@ -1685,14 +1585,14 @@
           <t>No invented facts</t>
         </is>
       </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>D – Bujji AI Property Assistant</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
+      <c r="B73" s="4" t="inlineStr">
         <is>
           <t>AI-02 Uncertainty &amp; escalation</t>
         </is>
@@ -1702,31 +1602,27 @@
           <t>Indicate insufficient data</t>
         </is>
       </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>D – Bujji AI Property Assistant</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>AI-02 Uncertainty &amp; escalation</t>
-        </is>
-      </c>
+      <c r="B74" s="5" t="n"/>
       <c r="C74" s="2" t="inlineStr">
         <is>
           <t>Bounded response; offer escalation</t>
         </is>
       </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>D – Bujji AI Property Assistant</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
+      <c r="B75" s="4" t="inlineStr">
         <is>
           <t>AI-03 Guardrails</t>
         </is>
@@ -1736,31 +1632,27 @@
           <t>Legal/financial disclaimers</t>
         </is>
       </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>D – Bujji AI Property Assistant</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>AI-03 Guardrails</t>
-        </is>
-      </c>
+      <c r="B76" s="5" t="n"/>
       <c r="C76" s="2" t="inlineStr">
         <is>
           <t>Red-team/UAT verification</t>
         </is>
       </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>D – Bujji AI Property Assistant</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
+      <c r="B77" s="4" t="inlineStr">
         <is>
           <t>AI-04 Telemetry</t>
         </is>
@@ -1770,31 +1662,27 @@
           <t>Capture latency, failure, feedback, source IDs</t>
         </is>
       </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>D – Bujji AI Property Assistant</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>AI-04 Telemetry</t>
-        </is>
-      </c>
+      <c r="B78" s="5" t="n"/>
       <c r="C78" s="2" t="inlineStr">
         <is>
           <t>Privacy-safe logs; ops can inspect failed/low-rated sessions</t>
         </is>
       </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>D – Bujji AI Property Assistant</t>
-        </is>
-      </c>
-      <c r="B79" s="2" t="inlineStr">
+      <c r="B79" s="4" t="inlineStr">
         <is>
           <t>AI-05 Version control</t>
         </is>
@@ -1804,31 +1692,27 @@
           <t>Version prompt/model/config</t>
         </is>
       </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>D – Bujji AI Property Assistant</t>
-        </is>
-      </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>AI-05 Version control</t>
-        </is>
-      </c>
+      <c r="B80" s="5" t="n"/>
       <c r="C80" s="2" t="inlineStr">
         <is>
           <t>Trace responses to deployed version</t>
         </is>
       </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="inlineStr">
-        <is>
-          <t>D – Bujji AI Property Assistant</t>
-        </is>
-      </c>
-      <c r="B81" s="2" t="inlineStr">
+      <c r="B81" s="4" t="inlineStr">
         <is>
           <t>AI-06 Lead routing</t>
         </is>
@@ -1838,31 +1722,27 @@
           <t>Create lead/service request with consent</t>
         </is>
       </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>D – Bujji AI Property Assistant</t>
-        </is>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>AI-06 Lead routing</t>
-        </is>
-      </c>
+      <c r="B82" s="5" t="n"/>
       <c r="C82" s="2" t="inlineStr">
         <is>
           <t>Include intent summary &amp; property/project ID</t>
         </is>
       </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="inlineStr">
-        <is>
-          <t>D – Bujji AI Property Assistant</t>
-        </is>
-      </c>
-      <c r="B83" s="2" t="inlineStr">
+      <c r="B83" s="4" t="inlineStr">
         <is>
           <t>AI-07 Memory/personalization</t>
         </is>
@@ -1872,31 +1752,33 @@
           <t>Retain preferences &amp; prior context with consent</t>
         </is>
       </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>D – Bujji AI Property Assistant</t>
-        </is>
-      </c>
-      <c r="B84" s="2" t="inlineStr">
-        <is>
-          <t>AI-07 Memory/personalization</t>
-        </is>
-      </c>
+      <c r="A84" s="5" t="n"/>
+      <c r="B84" s="5" t="n"/>
       <c r="C84" s="2" t="inlineStr">
         <is>
           <t>Avoid repeated questions</t>
         </is>
       </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="85">
-      <c r="A85" s="3" t="inlineStr">
+      <c r="A85" s="6" t="inlineStr">
         <is>
           <t>E – K-Report &amp; Legal Verification</t>
         </is>
       </c>
-      <c r="B85" s="3" t="inlineStr">
+      <c r="B85" s="6" t="inlineStr">
         <is>
           <t>KR-01 K-Report generation</t>
         </is>
@@ -1906,14 +1788,14 @@
           <t>Sections: property, ownership, registration, regulatory, location, risk/status</t>
         </is>
       </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" s="3" t="inlineStr">
-        <is>
-          <t>E – K-Report &amp; Legal Verification</t>
-        </is>
-      </c>
-      <c r="B86" s="3" t="inlineStr">
+      <c r="B86" s="6" t="inlineStr">
         <is>
           <t>KR-01 K-Report generation</t>
         </is>
@@ -1923,14 +1805,14 @@
           <t>Mark missing evidence as unavailable/not verified</t>
         </is>
       </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" s="3" t="inlineStr">
-        <is>
-          <t>E – K-Report &amp; Legal Verification</t>
-        </is>
-      </c>
-      <c r="B87" s="3" t="inlineStr">
+      <c r="B87" s="6" t="inlineStr">
         <is>
           <t>KR-02 Evidence tracking</t>
         </is>
@@ -1940,31 +1822,27 @@
           <t>Record source, date, verification status</t>
         </is>
       </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" s="3" t="inlineStr">
-        <is>
-          <t>E – K-Report &amp; Legal Verification</t>
-        </is>
-      </c>
-      <c r="B88" s="3" t="inlineStr">
-        <is>
-          <t>KR-02 Evidence tracking</t>
-        </is>
-      </c>
+      <c r="B88" s="5" t="n"/>
       <c r="C88" s="3" t="inlineStr">
         <is>
           <t>Distinguish user-provided / system-fetched / professionally verified</t>
         </is>
       </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" s="3" t="inlineStr">
-        <is>
-          <t>E – K-Report &amp; Legal Verification</t>
-        </is>
-      </c>
-      <c r="B89" s="3" t="inlineStr">
+      <c r="B89" s="6" t="inlineStr">
         <is>
           <t>KR-03 Legal-verification case</t>
         </is>
@@ -1974,31 +1852,27 @@
           <t>Create case with owner/partner, SLA, checklist</t>
         </is>
       </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" s="3" t="inlineStr">
-        <is>
-          <t>E – K-Report &amp; Legal Verification</t>
-        </is>
-      </c>
-      <c r="B90" s="3" t="inlineStr">
-        <is>
-          <t>KR-03 Legal-verification case</t>
-        </is>
-      </c>
+      <c r="B90" s="5" t="n"/>
       <c r="C90" s="3" t="inlineStr">
         <is>
           <t>Track request → report delivery with timestamps</t>
         </is>
       </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" s="3" t="inlineStr">
-        <is>
-          <t>E – K-Report &amp; Legal Verification</t>
-        </is>
-      </c>
-      <c r="B91" s="3" t="inlineStr">
+      <c r="B91" s="6" t="inlineStr">
         <is>
           <t>KR-04 Document access control</t>
         </is>
@@ -2008,31 +1882,27 @@
           <t>Restrict view/download to authorized roles</t>
         </is>
       </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" s="3" t="inlineStr">
-        <is>
-          <t>E – K-Report &amp; Legal Verification</t>
-        </is>
-      </c>
-      <c r="B92" s="3" t="inlineStr">
-        <is>
-          <t>KR-04 Document access control</t>
-        </is>
-      </c>
+      <c r="B92" s="5" t="n"/>
       <c r="C92" s="3" t="inlineStr">
         <is>
           <t>Log access</t>
         </is>
       </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="3" t="inlineStr">
-        <is>
-          <t>E – K-Report &amp; Legal Verification</t>
-        </is>
-      </c>
-      <c r="B93" s="3" t="inlineStr">
+      <c r="B93" s="6" t="inlineStr">
         <is>
           <t>KR-05 Legal opinion separation</t>
         </is>
@@ -2042,14 +1912,14 @@
           <t>Label automated output as not legal opinion unless professionally signed</t>
         </is>
       </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" s="3" t="inlineStr">
-        <is>
-          <t>E – K-Report &amp; Legal Verification</t>
-        </is>
-      </c>
-      <c r="B94" s="3" t="inlineStr">
+      <c r="B94" s="6" t="inlineStr">
         <is>
           <t>KR-06 Report versioning</t>
         </is>
@@ -2059,31 +1929,33 @@
           <t>Regenerate on source change</t>
         </is>
       </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="3" t="inlineStr">
-        <is>
-          <t>E – K-Report &amp; Legal Verification</t>
-        </is>
-      </c>
-      <c r="B95" s="3" t="inlineStr">
-        <is>
-          <t>KR-06 Report versioning</t>
-        </is>
-      </c>
+      <c r="A95" s="5" t="n"/>
+      <c r="B95" s="5" t="n"/>
       <c r="C95" s="3" t="inlineStr">
         <is>
           <t>Keep prior versions; flag current</t>
         </is>
       </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="inlineStr">
+      <c r="A96" s="4" t="inlineStr">
         <is>
           <t>F – MySecure</t>
         </is>
       </c>
-      <c r="B96" s="2" t="inlineStr">
+      <c r="B96" s="4" t="inlineStr">
         <is>
           <t>MS-01 Plan enrollment</t>
         </is>
@@ -2093,14 +1965,14 @@
           <t>Capture property, authorized contacts, plan, consent, special instructions</t>
         </is>
       </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="inlineStr">
-        <is>
-          <t>F – MySecure</t>
-        </is>
-      </c>
-      <c r="B97" s="2" t="inlineStr">
+      <c r="B97" s="4" t="inlineStr">
         <is>
           <t>MS-01 Plan enrollment</t>
         </is>
@@ -2110,14 +1982,14 @@
           <t>Access/contact instructions</t>
         </is>
       </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>F – MySecure</t>
-        </is>
-      </c>
-      <c r="B98" s="2" t="inlineStr">
+      <c r="B98" s="4" t="inlineStr">
         <is>
           <t>MS-02 Inspection scheduling</t>
         </is>
@@ -2127,31 +1999,27 @@
           <t>Schedule recurring visits per plan</t>
         </is>
       </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="inlineStr">
-        <is>
-          <t>F – MySecure</t>
-        </is>
-      </c>
-      <c r="B99" s="2" t="inlineStr">
-        <is>
-          <t>MS-02 Inspection scheduling</t>
-        </is>
-      </c>
+      <c r="B99" s="5" t="n"/>
       <c r="C99" s="2" t="inlineStr">
         <is>
           <t>Show upcoming/overdue with field owner</t>
         </is>
       </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>F – MySecure</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="inlineStr">
+      <c r="B100" s="4" t="inlineStr">
         <is>
           <t>MS-03 Field inspection</t>
         </is>
@@ -2161,31 +2029,27 @@
           <t>Timestamped photos/video, checklist, notes</t>
         </is>
       </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="inlineStr">
-        <is>
-          <t>F – MySecure</t>
-        </is>
-      </c>
-      <c r="B101" s="2" t="inlineStr">
-        <is>
-          <t>MS-03 Field inspection</t>
-        </is>
-      </c>
+      <c r="B101" s="5" t="n"/>
       <c r="C101" s="2" t="inlineStr">
         <is>
           <t>Block closure on incomplete checklist without exception reason</t>
         </is>
       </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>F – MySecure</t>
-        </is>
-      </c>
-      <c r="B102" s="2" t="inlineStr">
+      <c r="B102" s="4" t="inlineStr">
         <is>
           <t>MS-04 Owner report &amp; alerts</t>
         </is>
@@ -2195,31 +2059,27 @@
           <t>Post-inspection owner report</t>
         </is>
       </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t>F – MySecure</t>
-        </is>
-      </c>
-      <c r="B103" s="2" t="inlineStr">
-        <is>
-          <t>MS-04 Owner report &amp; alerts</t>
-        </is>
-      </c>
+      <c r="B103" s="5" t="n"/>
       <c r="C103" s="2" t="inlineStr">
         <is>
           <t>Critical-issue escalation</t>
         </is>
       </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>F – MySecure</t>
-        </is>
-      </c>
-      <c r="B104" s="2" t="inlineStr">
+      <c r="B104" s="4" t="inlineStr">
         <is>
           <t>MS-05 Plan history &amp; status</t>
         </is>
@@ -2229,31 +2089,27 @@
           <t>Maintain payments/service period</t>
         </is>
       </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="inlineStr">
-        <is>
-          <t>F – MySecure</t>
-        </is>
-      </c>
-      <c r="B105" s="2" t="inlineStr">
-        <is>
-          <t>MS-05 Plan history &amp; status</t>
-        </is>
-      </c>
+      <c r="B105" s="5" t="n"/>
       <c r="C105" s="2" t="inlineStr">
         <is>
           <t>Active/expired/suspended state &amp; renewal date</t>
         </is>
       </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>F – MySecure</t>
-        </is>
-      </c>
-      <c r="B106" s="2" t="inlineStr">
+      <c r="B106" s="4" t="inlineStr">
         <is>
           <t>MS-06 Maintenance/vendor tasks</t>
         </is>
@@ -2263,31 +2119,27 @@
           <t>Track separately from inspection</t>
         </is>
       </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>F – MySecure</t>
-        </is>
-      </c>
-      <c r="B107" s="2" t="inlineStr">
-        <is>
-          <t>MS-06 Maintenance/vendor tasks</t>
-        </is>
-      </c>
+      <c r="B107" s="5" t="n"/>
       <c r="C107" s="2" t="inlineStr">
         <is>
           <t>Owner approval, cost, status</t>
         </is>
       </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>F – MySecure</t>
-        </is>
-      </c>
-      <c r="B108" s="2" t="inlineStr">
+      <c r="B108" s="4" t="inlineStr">
         <is>
           <t>MS-07 Area alerts</t>
         </is>
@@ -2297,31 +2149,33 @@
           <t>Alerts on developments/infra/significant changes</t>
         </is>
       </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="inlineStr">
-        <is>
-          <t>F – MySecure</t>
-        </is>
-      </c>
-      <c r="B109" s="2" t="inlineStr">
-        <is>
-          <t>MS-07 Area alerts</t>
-        </is>
-      </c>
+      <c r="A109" s="5" t="n"/>
+      <c r="B109" s="5" t="n"/>
       <c r="C109" s="2" t="inlineStr">
         <is>
           <t>Owner dashboard &amp; notification channels</t>
         </is>
       </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="110">
-      <c r="A110" s="3" t="inlineStr">
+      <c r="A110" s="6" t="inlineStr">
         <is>
           <t>G – KONU Buddies / Agent Network</t>
         </is>
       </c>
-      <c r="B110" s="3" t="inlineStr">
+      <c r="B110" s="6" t="inlineStr">
         <is>
           <t>KB-01 Buddy application</t>
         </is>
@@ -2331,14 +2185,14 @@
           <t>Capture identity, contact, coverage, experience, documents</t>
         </is>
       </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="111">
-      <c r="A111" s="3" t="inlineStr">
-        <is>
-          <t>G – KONU Buddies / Agent Network</t>
-        </is>
-      </c>
-      <c r="B111" s="3" t="inlineStr">
+      <c r="B111" s="6" t="inlineStr">
         <is>
           <t>KB-01 Buddy application</t>
         </is>
@@ -2348,14 +2202,14 @@
           <t>Block activation if verification incomplete</t>
         </is>
       </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="112">
-      <c r="A112" s="3" t="inlineStr">
-        <is>
-          <t>G – KONU Buddies / Agent Network</t>
-        </is>
-      </c>
-      <c r="B112" s="3" t="inlineStr">
+      <c r="B112" s="6" t="inlineStr">
         <is>
           <t>KB-02 Admin approval</t>
         </is>
@@ -2365,31 +2219,27 @@
           <t>Approve/reject/suspend with reason</t>
         </is>
       </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="113">
-      <c r="A113" s="3" t="inlineStr">
-        <is>
-          <t>G – KONU Buddies / Agent Network</t>
-        </is>
-      </c>
-      <c r="B113" s="3" t="inlineStr">
-        <is>
-          <t>KB-02 Admin approval</t>
-        </is>
-      </c>
+      <c r="B113" s="5" t="n"/>
       <c r="C113" s="3" t="inlineStr">
         <is>
           <t>Audit log; no leads to inactive/suspended</t>
         </is>
       </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="114">
-      <c r="A114" s="3" t="inlineStr">
-        <is>
-          <t>G – KONU Buddies / Agent Network</t>
-        </is>
-      </c>
-      <c r="B114" s="3" t="inlineStr">
+      <c r="B114" s="6" t="inlineStr">
         <is>
           <t>KB-03 Lead assignment</t>
         </is>
@@ -2399,31 +2249,27 @@
           <t>Assign owner, SLA, status, handoff notes</t>
         </is>
       </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="115">
-      <c r="A115" s="3" t="inlineStr">
-        <is>
-          <t>G – KONU Buddies / Agent Network</t>
-        </is>
-      </c>
-      <c r="B115" s="3" t="inlineStr">
-        <is>
-          <t>KB-03 Lead assignment</t>
-        </is>
-      </c>
+      <c r="B115" s="5" t="n"/>
       <c r="C115" s="3" t="inlineStr">
         <is>
           <t>Track timestamps &amp; next action</t>
         </is>
       </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="116">
-      <c r="A116" s="3" t="inlineStr">
-        <is>
-          <t>G – KONU Buddies / Agent Network</t>
-        </is>
-      </c>
-      <c r="B116" s="3" t="inlineStr">
+      <c r="B116" s="6" t="inlineStr">
         <is>
           <t>KB-04 Mandate/transaction workflow</t>
         </is>
@@ -2433,31 +2279,27 @@
           <t>Track property/customer &amp; milestones</t>
         </is>
       </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="117">
-      <c r="A117" s="3" t="inlineStr">
-        <is>
-          <t>G – KONU Buddies / Agent Network</t>
-        </is>
-      </c>
-      <c r="B117" s="3" t="inlineStr">
-        <is>
-          <t>KB-04 Mandate/transaction workflow</t>
-        </is>
-      </c>
+      <c r="B117" s="5" t="n"/>
       <c r="C117" s="3" t="inlineStr">
         <is>
           <t>Audit changes; closed-lost reason</t>
         </is>
       </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="118">
-      <c r="A118" s="3" t="inlineStr">
-        <is>
-          <t>G – KONU Buddies / Agent Network</t>
-        </is>
-      </c>
-      <c r="B118" s="3" t="inlineStr">
+      <c r="B118" s="6" t="inlineStr">
         <is>
           <t>KB-05 Quality &amp; feedback</t>
         </is>
@@ -2467,31 +2309,27 @@
           <t>Link metrics/feedback to Buddy profile</t>
         </is>
       </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="119">
-      <c r="A119" s="3" t="inlineStr">
-        <is>
-          <t>G – KONU Buddies / Agent Network</t>
-        </is>
-      </c>
-      <c r="B119" s="3" t="inlineStr">
-        <is>
-          <t>KB-05 Quality &amp; feedback</t>
-        </is>
-      </c>
+      <c r="B119" s="5" t="n"/>
       <c r="C119" s="3" t="inlineStr">
         <is>
           <t>Performance reporting</t>
         </is>
       </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="120">
-      <c r="A120" s="3" t="inlineStr">
-        <is>
-          <t>G – KONU Buddies / Agent Network</t>
-        </is>
-      </c>
-      <c r="B120" s="3" t="inlineStr">
+      <c r="B120" s="6" t="inlineStr">
         <is>
           <t>KB-06 Commission policy</t>
         </is>
@@ -2501,31 +2339,27 @@
           <t>Configurable rule/reference recorded</t>
         </is>
       </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="121">
-      <c r="A121" s="3" t="inlineStr">
-        <is>
-          <t>G – KONU Buddies / Agent Network</t>
-        </is>
-      </c>
-      <c r="B121" s="3" t="inlineStr">
-        <is>
-          <t>KB-06 Commission policy</t>
-        </is>
-      </c>
+      <c r="B121" s="5" t="n"/>
       <c r="C121" s="3" t="inlineStr">
         <is>
           <t>No hardcoded rates; settlement out of scope</t>
         </is>
       </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="122">
-      <c r="A122" s="3" t="inlineStr">
-        <is>
-          <t>G – KONU Buddies / Agent Network</t>
-        </is>
-      </c>
-      <c r="B122" s="3" t="inlineStr">
+      <c r="B122" s="6" t="inlineStr">
         <is>
           <t>KB-07 Location-based matching</t>
         </is>
@@ -2535,31 +2369,33 @@
           <t>Match by location, service area, proximity, availability</t>
         </is>
       </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="123">
-      <c r="A123" s="3" t="inlineStr">
-        <is>
-          <t>G – KONU Buddies / Agent Network</t>
-        </is>
-      </c>
-      <c r="B123" s="3" t="inlineStr">
-        <is>
-          <t>KB-07 Location-based matching</t>
-        </is>
-      </c>
+      <c r="A123" s="5" t="n"/>
+      <c r="B123" s="5" t="n"/>
       <c r="C123" s="3" t="inlineStr">
         <is>
           <t>Accept lead; single accountable owner; track status</t>
         </is>
       </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="inlineStr">
+      <c r="A124" s="4" t="inlineStr">
         <is>
           <t>H – Developer Services, CRM &amp; Growth Analytics</t>
         </is>
       </c>
-      <c r="B124" s="2" t="inlineStr">
+      <c r="B124" s="4" t="inlineStr">
         <is>
           <t>DEV-01 Developer/project onboarding</t>
         </is>
@@ -2569,14 +2405,14 @@
           <t>Capture company, project, RERA IDs, location, inventory, contacts</t>
         </is>
       </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="inlineStr">
-        <is>
-          <t>H – Developer Services, CRM &amp; Growth Analytics</t>
-        </is>
-      </c>
-      <c r="B125" s="2" t="inlineStr">
+      <c r="B125" s="4" t="inlineStr">
         <is>
           <t>DEV-01 Developer/project onboarding</t>
         </is>
@@ -2586,14 +2422,14 @@
           <t>Admin verification before verified status</t>
         </is>
       </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="inlineStr">
-        <is>
-          <t>H – Developer Services, CRM &amp; Growth Analytics</t>
-        </is>
-      </c>
-      <c r="B126" s="2" t="inlineStr">
+      <c r="B126" s="4" t="inlineStr">
         <is>
           <t>DEV-02 Project pages</t>
         </is>
@@ -2603,31 +2439,27 @@
           <t>Inventory/media/amenity/location content</t>
         </is>
       </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="inlineStr">
-        <is>
-          <t>H – Developer Services, CRM &amp; Growth Analytics</t>
-        </is>
-      </c>
-      <c r="B127" s="2" t="inlineStr">
-        <is>
-          <t>DEV-02 Project pages</t>
-        </is>
-      </c>
+      <c r="B127" s="5" t="n"/>
       <c r="C127" s="2" t="inlineStr">
         <is>
           <t>Versioned, traceable to authorized source</t>
         </is>
       </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="inlineStr">
-        <is>
-          <t>H – Developer Services, CRM &amp; Growth Analytics</t>
-        </is>
-      </c>
-      <c r="B128" s="2" t="inlineStr">
+      <c r="B128" s="4" t="inlineStr">
         <is>
           <t>DEV-03 Lead capture</t>
         </is>
@@ -2637,31 +2469,27 @@
           <t>Preserve project, channel/campaign, consent</t>
         </is>
       </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="inlineStr">
-        <is>
-          <t>H – Developer Services, CRM &amp; Growth Analytics</t>
-        </is>
-      </c>
-      <c r="B129" s="2" t="inlineStr">
-        <is>
-          <t>DEV-03 Lead capture</t>
-        </is>
-      </c>
+      <c r="B129" s="5" t="n"/>
       <c r="C129" s="2" t="inlineStr">
         <is>
           <t>Deduplicate per approved rules</t>
         </is>
       </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="inlineStr">
-        <is>
-          <t>H – Developer Services, CRM &amp; Growth Analytics</t>
-        </is>
-      </c>
-      <c r="B130" s="2" t="inlineStr">
+      <c r="B130" s="4" t="inlineStr">
         <is>
           <t>DEV-04 Lead feedback loop</t>
         </is>
@@ -2671,31 +2499,27 @@
           <t>Sales/CRM status flows back</t>
         </is>
       </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="inlineStr">
-        <is>
-          <t>H – Developer Services, CRM &amp; Growth Analytics</t>
-        </is>
-      </c>
-      <c r="B131" s="2" t="inlineStr">
-        <is>
-          <t>DEV-04 Lead feedback loop</t>
-        </is>
-      </c>
+      <c r="B131" s="5" t="n"/>
       <c r="C131" s="2" t="inlineStr">
         <is>
           <t>Report lead volume &amp; downstream status</t>
         </is>
       </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="inlineStr">
-        <is>
-          <t>H – Developer Services, CRM &amp; Growth Analytics</t>
-        </is>
-      </c>
-      <c r="B132" s="2" t="inlineStr">
+      <c r="B132" s="4" t="inlineStr">
         <is>
           <t>DEV-05 Funnel analytics</t>
         </is>
@@ -2705,31 +2529,27 @@
           <t>Document event taxonomy</t>
         </is>
       </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="inlineStr">
-        <is>
-          <t>H – Developer Services, CRM &amp; Growth Analytics</t>
-        </is>
-      </c>
-      <c r="B133" s="2" t="inlineStr">
-        <is>
-          <t>DEV-05 Funnel analytics</t>
-        </is>
-      </c>
+      <c r="B133" s="5" t="n"/>
       <c r="C133" s="2" t="inlineStr">
         <is>
           <t>QA acquisition → engagement → conversion events</t>
         </is>
       </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="inlineStr">
-        <is>
-          <t>H – Developer Services, CRM &amp; Growth Analytics</t>
-        </is>
-      </c>
-      <c r="B134" s="2" t="inlineStr">
+      <c r="B134" s="4" t="inlineStr">
         <is>
           <t>DEV-06 Commercial model config</t>
         </is>
@@ -2739,31 +2559,27 @@
           <t>Configurable pricing/ACV/success-fee</t>
         </is>
       </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="inlineStr">
-        <is>
-          <t>H – Developer Services, CRM &amp; Growth Analytics</t>
-        </is>
-      </c>
-      <c r="B135" s="2" t="inlineStr">
-        <is>
-          <t>DEV-06 Commercial model config</t>
-        </is>
-      </c>
+      <c r="B135" s="5" t="n"/>
       <c r="C135" s="2" t="inlineStr">
         <is>
           <t>No unapproved assumptions in logic</t>
         </is>
       </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="inlineStr">
-        <is>
-          <t>H – Developer Services, CRM &amp; Growth Analytics</t>
-        </is>
-      </c>
-      <c r="B136" s="2" t="inlineStr">
+      <c r="B136" s="4" t="inlineStr">
         <is>
           <t>DEV-07 KONU Custom CRM</t>
         </is>
@@ -2773,48 +2589,45 @@
           <t>Customer, property, lead, Buddy, developer, transaction journeys</t>
         </is>
       </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="inlineStr">
-        <is>
-          <t>H – Developer Services, CRM &amp; Growth Analytics</t>
-        </is>
-      </c>
-      <c r="B137" s="2" t="inlineStr">
-        <is>
-          <t>DEV-07 KONU Custom CRM</t>
-        </is>
-      </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
           <t>Unified history, integrations, reporting</t>
         </is>
       </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="inlineStr">
-        <is>
-          <t>H – Developer Services, CRM &amp; Growth Analytics</t>
-        </is>
-      </c>
-      <c r="B138" s="2" t="inlineStr">
-        <is>
-          <t>DEV-07 KONU Custom CRM</t>
-        </is>
-      </c>
+      <c r="A138" s="5" t="n"/>
+      <c r="B138" s="5" t="n"/>
       <c r="C138" s="2" t="inlineStr">
         <is>
           <t>Transition from third-party CRM</t>
         </is>
       </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="139">
-      <c r="A139" s="3" t="inlineStr">
+      <c r="A139" s="6" t="inlineStr">
         <is>
           <t>I – Admin, Data Ops, Notifications &amp; Platform Controls</t>
         </is>
       </c>
-      <c r="B139" s="3" t="inlineStr">
+      <c r="B139" s="6" t="inlineStr">
         <is>
           <t>ADM-01 Role-based access</t>
         </is>
@@ -2824,14 +2637,14 @@
           <t>Separate content, ops, QA, service, super-admin roles</t>
         </is>
       </c>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="140">
-      <c r="A140" s="3" t="inlineStr">
-        <is>
-          <t>I – Admin, Data Ops, Notifications &amp; Platform Controls</t>
-        </is>
-      </c>
-      <c r="B140" s="3" t="inlineStr">
+      <c r="B140" s="6" t="inlineStr">
         <is>
           <t>ADM-01 Role-based access</t>
         </is>
@@ -2841,14 +2654,14 @@
           <t>Permission testing</t>
         </is>
       </c>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="141">
-      <c r="A141" s="3" t="inlineStr">
-        <is>
-          <t>I – Admin, Data Ops, Notifications &amp; Platform Controls</t>
-        </is>
-      </c>
-      <c r="B141" s="3" t="inlineStr">
+      <c r="B141" s="6" t="inlineStr">
         <is>
           <t>ADM-02 Master data &amp; exceptions</t>
         </is>
@@ -2858,31 +2671,27 @@
           <t>Manage master data, verification status, exception queues</t>
         </is>
       </c>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="142">
-      <c r="A142" s="3" t="inlineStr">
-        <is>
-          <t>I – Admin, Data Ops, Notifications &amp; Platform Controls</t>
-        </is>
-      </c>
-      <c r="B142" s="3" t="inlineStr">
-        <is>
-          <t>ADM-02 Master data &amp; exceptions</t>
-        </is>
-      </c>
+      <c r="B142" s="5" t="n"/>
       <c r="C142" s="3" t="inlineStr">
         <is>
           <t>Audited; no direct DB edits</t>
         </is>
       </c>
+      <c r="D142" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="143">
-      <c r="A143" s="3" t="inlineStr">
-        <is>
-          <t>I – Admin, Data Ops, Notifications &amp; Platform Controls</t>
-        </is>
-      </c>
-      <c r="B143" s="3" t="inlineStr">
+      <c r="B143" s="6" t="inlineStr">
         <is>
           <t>ADM-03 Notification service</t>
         </is>
@@ -2892,31 +2701,27 @@
           <t>Transactional messages &amp; delivery status</t>
         </is>
       </c>
+      <c r="D143" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="144">
-      <c r="A144" s="3" t="inlineStr">
-        <is>
-          <t>I – Admin, Data Ops, Notifications &amp; Platform Controls</t>
-        </is>
-      </c>
-      <c r="B144" s="3" t="inlineStr">
-        <is>
-          <t>ADM-03 Notification service</t>
-        </is>
-      </c>
+      <c r="B144" s="5" t="n"/>
       <c r="C144" s="3" t="inlineStr">
         <is>
           <t>Log/retry failures</t>
         </is>
       </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="145">
-      <c r="A145" s="3" t="inlineStr">
-        <is>
-          <t>I – Admin, Data Ops, Notifications &amp; Platform Controls</t>
-        </is>
-      </c>
-      <c r="B145" s="3" t="inlineStr">
+      <c r="B145" s="6" t="inlineStr">
         <is>
           <t>ADM-04 Pipeline status</t>
         </is>
@@ -2926,31 +2731,27 @@
           <t>Show last success, error, owner</t>
         </is>
       </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="146">
-      <c r="A146" s="3" t="inlineStr">
-        <is>
-          <t>I – Admin, Data Ops, Notifications &amp; Platform Controls</t>
-        </is>
-      </c>
-      <c r="B146" s="3" t="inlineStr">
-        <is>
-          <t>ADM-04 Pipeline status</t>
-        </is>
-      </c>
+      <c r="B146" s="5" t="n"/>
       <c r="C146" s="3" t="inlineStr">
         <is>
           <t>Identify stale/failed sources</t>
         </is>
       </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="147">
-      <c r="A147" s="3" t="inlineStr">
-        <is>
-          <t>I – Admin, Data Ops, Notifications &amp; Platform Controls</t>
-        </is>
-      </c>
-      <c r="B147" s="3" t="inlineStr">
+      <c r="B147" s="6" t="inlineStr">
         <is>
           <t>ADM-05 Audit trail</t>
         </is>
@@ -2960,14 +2761,14 @@
           <t>Actor/time/action history for critical entities</t>
         </is>
       </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="148">
-      <c r="A148" s="3" t="inlineStr">
-        <is>
-          <t>I – Admin, Data Ops, Notifications &amp; Platform Controls</t>
-        </is>
-      </c>
-      <c r="B148" s="3" t="inlineStr">
+      <c r="B148" s="6" t="inlineStr">
         <is>
           <t>ADM-06 Environment separation</t>
         </is>
@@ -2977,31 +2778,33 @@
           <t>Separate dev/test/prod config</t>
         </is>
       </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="149">
-      <c r="A149" s="3" t="inlineStr">
-        <is>
-          <t>I – Admin, Data Ops, Notifications &amp; Platform Controls</t>
-        </is>
-      </c>
-      <c r="B149" s="3" t="inlineStr">
-        <is>
-          <t>ADM-06 Environment separation</t>
-        </is>
-      </c>
+      <c r="A149" s="5" t="n"/>
+      <c r="B149" s="5" t="n"/>
       <c r="C149" s="3" t="inlineStr">
         <is>
           <t>Isolate production secrets</t>
         </is>
       </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="inlineStr">
+      <c r="A150" s="4" t="inlineStr">
         <is>
           <t>J – Customer Dashboard</t>
         </is>
       </c>
-      <c r="B150" s="2" t="inlineStr">
+      <c r="B150" s="4" t="inlineStr">
         <is>
           <t>CD-01 Property activity</t>
         </is>
@@ -3011,14 +2814,14 @@
           <t>Recently viewed</t>
         </is>
       </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="inlineStr">
-        <is>
-          <t>J – Customer Dashboard</t>
-        </is>
-      </c>
-      <c r="B151" s="2" t="inlineStr">
+      <c r="B151" s="4" t="inlineStr">
         <is>
           <t>CD-01 Property activity</t>
         </is>
@@ -3028,31 +2831,27 @@
           <t>Saved/interested</t>
         </is>
       </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="inlineStr">
-        <is>
-          <t>J – Customer Dashboard</t>
-        </is>
-      </c>
-      <c r="B152" s="2" t="inlineStr">
-        <is>
-          <t>CD-01 Property activity</t>
-        </is>
-      </c>
+      <c r="B152" s="5" t="n"/>
       <c r="C152" s="2" t="inlineStr">
         <is>
           <t>Rejected/not-interested</t>
         </is>
       </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="inlineStr">
-        <is>
-          <t>J – Customer Dashboard</t>
-        </is>
-      </c>
-      <c r="B153" s="2" t="inlineStr">
+      <c r="B153" s="4" t="inlineStr">
         <is>
           <t>CD-02 Analytics &amp; insights</t>
         </is>
@@ -3062,31 +2861,27 @@
           <t>Customer-level property analytics</t>
         </is>
       </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="inlineStr">
-        <is>
-          <t>J – Customer Dashboard</t>
-        </is>
-      </c>
-      <c r="B154" s="2" t="inlineStr">
-        <is>
-          <t>CD-02 Analytics &amp; insights</t>
-        </is>
-      </c>
+      <c r="B154" s="5" t="n"/>
       <c r="C154" s="2" t="inlineStr">
         <is>
           <t>Insights from activity, preferences, owned properties</t>
         </is>
       </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="inlineStr">
-        <is>
-          <t>J – Customer Dashboard</t>
-        </is>
-      </c>
-      <c r="B155" s="2" t="inlineStr">
+      <c r="B155" s="4" t="inlineStr">
         <is>
           <t>CD-03 New-match alerts</t>
         </is>
@@ -3096,31 +2891,27 @@
           <t>Alert on new property matching preferences</t>
         </is>
       </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="inlineStr">
-        <is>
-          <t>J – Customer Dashboard</t>
-        </is>
-      </c>
-      <c r="B156" s="2" t="inlineStr">
-        <is>
-          <t>CD-03 New-match alerts</t>
-        </is>
-      </c>
+      <c r="B156" s="5" t="n"/>
       <c r="C156" s="2" t="inlineStr">
         <is>
           <t>Card/notification with direct listing link</t>
         </is>
       </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="inlineStr">
-        <is>
-          <t>J – Customer Dashboard</t>
-        </is>
-      </c>
-      <c r="B157" s="2" t="inlineStr">
+      <c r="B157" s="4" t="inlineStr">
         <is>
           <t>CD-04 Service status</t>
         </is>
@@ -3130,31 +2921,27 @@
           <t>Active KONU services incl. MySecure</t>
         </is>
       </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="inlineStr">
-        <is>
-          <t>J – Customer Dashboard</t>
-        </is>
-      </c>
-      <c r="B158" s="2" t="inlineStr">
-        <is>
-          <t>CD-04 Service status</t>
-        </is>
-      </c>
+      <c r="B158" s="5" t="n"/>
       <c r="C158" s="2" t="inlineStr">
         <is>
           <t>Status, recent activity, next actions</t>
         </is>
       </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="inlineStr">
-        <is>
-          <t>J – Customer Dashboard</t>
-        </is>
-      </c>
-      <c r="B159" s="2" t="inlineStr">
+      <c r="B159" s="4" t="inlineStr">
         <is>
           <t>CD-05 Personalized updates</t>
         </is>
@@ -3164,26 +2951,107 @@
           <t>Notifications &amp; recommendations</t>
         </is>
       </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
     <row r="160">
-      <c r="A160" s="2" t="inlineStr">
-        <is>
-          <t>J – Customer Dashboard</t>
-        </is>
-      </c>
-      <c r="B160" s="2" t="inlineStr">
-        <is>
-          <t>CD-05 Personalized updates</t>
-        </is>
-      </c>
+      <c r="A160" s="5" t="n"/>
+      <c r="B160" s="5" t="n"/>
       <c r="C160" s="2" t="inlineStr">
         <is>
           <t>Important journey updates</t>
         </is>
       </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C160"/>
+  <autoFilter ref="A1:D160"/>
+  <mergeCells count="72">
+    <mergeCell ref="B122:B123"/>
+    <mergeCell ref="B155:B156"/>
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="A42:A55"/>
+    <mergeCell ref="B130:B131"/>
+    <mergeCell ref="A96:A109"/>
+    <mergeCell ref="B77:B78"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="B102:B103"/>
+    <mergeCell ref="A2:A19"/>
+    <mergeCell ref="A139:A149"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="B148:B149"/>
+    <mergeCell ref="B145:B146"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="B120:B121"/>
+    <mergeCell ref="A124:A138"/>
+    <mergeCell ref="B132:B133"/>
+    <mergeCell ref="B157:B158"/>
+    <mergeCell ref="B51:B53"/>
+    <mergeCell ref="B151:B152"/>
+    <mergeCell ref="B60:B61"/>
+    <mergeCell ref="B98:B99"/>
+    <mergeCell ref="B116:B117"/>
+    <mergeCell ref="B69:B70"/>
+    <mergeCell ref="A85:A95"/>
+    <mergeCell ref="B63:B65"/>
+    <mergeCell ref="B143:B144"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="A150:A160"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="B128:B129"/>
+    <mergeCell ref="A56:A70"/>
+    <mergeCell ref="B118:B119"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="B87:B88"/>
+    <mergeCell ref="B83:B84"/>
+    <mergeCell ref="B112:B113"/>
+    <mergeCell ref="A20:A41"/>
+    <mergeCell ref="B108:B109"/>
+    <mergeCell ref="A110:A123"/>
+    <mergeCell ref="B89:B90"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="B106:B107"/>
+    <mergeCell ref="B114:B115"/>
+    <mergeCell ref="B136:B138"/>
+    <mergeCell ref="B79:B80"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="A71:A84"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B75:B76"/>
+    <mergeCell ref="B126:B127"/>
+    <mergeCell ref="B141:B142"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="B104:B105"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="B94:B95"/>
+    <mergeCell ref="B91:B92"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="B134:B135"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="B159:B160"/>
+    <mergeCell ref="B153:B154"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="B100:B101"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D160" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Not Started,In Progress,Done,Blocked"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Data Science sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01319BznfEv5w8UGSo5VivdJ
</commit_message>
<xml_diff>
--- a/docs/KONU_BRD_Functionalities.xlsx
+++ b/docs/KONU_BRD_Functionalities.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="KONU Functionalities" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Data Science" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'KONU Functionalities'!$A$1:$D$160</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Data Science'!$A$1:$D$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -61,7 +63,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -83,11 +85,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -103,6 +111,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -502,7 +516,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>NFR – Platform Requirements</t>
         </is>
@@ -512,7 +526,7 @@
           <t>NFR-01 Availability</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Monitor launch-critical flows</t>
         </is>
@@ -541,7 +555,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>NFR-02 Performance</t>
         </is>
@@ -571,7 +585,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>NFR-03 Security</t>
         </is>
@@ -613,7 +627,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>NFR-04 Privacy</t>
         </is>
@@ -655,7 +669,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>NFR-05 Observability</t>
         </is>
@@ -702,7 +716,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>NFR-07 Accessibility</t>
         </is>
@@ -744,7 +758,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>NFR-08 Scalability</t>
         </is>
@@ -775,7 +789,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>A – Core Listings, Search &amp; Property Detail</t>
         </is>
@@ -814,7 +828,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>CL-02 Property card/detail</t>
         </is>
@@ -856,7 +870,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>CL-03 Map/list sync</t>
         </is>
@@ -886,7 +900,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>CL-04 Save/favorite</t>
         </is>
@@ -928,7 +942,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>CL-05 Lead/service CTA</t>
         </is>
@@ -958,7 +972,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>CL-06 Admin listing management</t>
         </is>
@@ -1000,7 +1014,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>CL-07 Duplicate/stale flagging</t>
         </is>
@@ -1030,7 +1044,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>CL-08 Personalized discovery</t>
         </is>
@@ -1060,7 +1074,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>CL-09 Engagement metrics</t>
         </is>
@@ -1103,7 +1117,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+      <c r="A42" s="7" t="inlineStr">
         <is>
           <t>B – GIS &amp; Hyperlocal Intelligence</t>
         </is>
@@ -1142,7 +1156,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B44" s="7" t="inlineStr">
         <is>
           <t>GIS-02 Infrastructure/POI layers</t>
         </is>
@@ -1184,7 +1198,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="4" t="inlineStr">
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>GIS-03 Boundary overlays</t>
         </is>
@@ -1214,7 +1228,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="B49" s="4" t="inlineStr">
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>GIS-04 Graceful API failure</t>
         </is>
@@ -1244,7 +1258,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B51" s="7" t="inlineStr">
         <is>
           <t>GIS-05 Spatial dataset updates</t>
         </is>
@@ -1286,7 +1300,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="B54" s="4" t="inlineStr">
+      <c r="B54" s="7" t="inlineStr">
         <is>
           <t>GIS-06 Nearby updates</t>
         </is>
@@ -1317,7 +1331,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="inlineStr">
+      <c r="A56" s="8" t="inlineStr">
         <is>
           <t>C – Kestimate</t>
         </is>
@@ -1356,7 +1370,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="B58" s="6" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>KE-02 Range/confidence</t>
         </is>
@@ -1386,7 +1400,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="B60" s="6" t="inlineStr">
+      <c r="B60" s="8" t="inlineStr">
         <is>
           <t>KE-03 Audit traceability</t>
         </is>
@@ -1433,7 +1447,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="B63" s="6" t="inlineStr">
+      <c r="B63" s="8" t="inlineStr">
         <is>
           <t>KE-05 Data-quality rules</t>
         </is>
@@ -1475,7 +1489,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="B66" s="6" t="inlineStr">
+      <c r="B66" s="8" t="inlineStr">
         <is>
           <t>KE-06 Monitoring</t>
         </is>
@@ -1522,7 +1536,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="B69" s="6" t="inlineStr">
+      <c r="B69" s="8" t="inlineStr">
         <is>
           <t>KE-08 GIS-driven refresh</t>
         </is>
@@ -1553,7 +1567,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="4" t="inlineStr">
+      <c r="A71" s="7" t="inlineStr">
         <is>
           <t>D – Bujji AI Property Assistant</t>
         </is>
@@ -1592,7 +1606,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="B73" s="4" t="inlineStr">
+      <c r="B73" s="7" t="inlineStr">
         <is>
           <t>AI-02 Uncertainty &amp; escalation</t>
         </is>
@@ -1622,7 +1636,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="B75" s="4" t="inlineStr">
+      <c r="B75" s="7" t="inlineStr">
         <is>
           <t>AI-03 Guardrails</t>
         </is>
@@ -1652,7 +1666,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="B77" s="4" t="inlineStr">
+      <c r="B77" s="7" t="inlineStr">
         <is>
           <t>AI-04 Telemetry</t>
         </is>
@@ -1682,7 +1696,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="B79" s="4" t="inlineStr">
+      <c r="B79" s="7" t="inlineStr">
         <is>
           <t>AI-05 Version control</t>
         </is>
@@ -1712,7 +1726,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="B81" s="4" t="inlineStr">
+      <c r="B81" s="7" t="inlineStr">
         <is>
           <t>AI-06 Lead routing</t>
         </is>
@@ -1742,7 +1756,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="B83" s="4" t="inlineStr">
+      <c r="B83" s="7" t="inlineStr">
         <is>
           <t>AI-07 Memory/personalization</t>
         </is>
@@ -1773,7 +1787,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="6" t="inlineStr">
+      <c r="A85" s="8" t="inlineStr">
         <is>
           <t>E – K-Report &amp; Legal Verification</t>
         </is>
@@ -1812,7 +1826,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="B87" s="6" t="inlineStr">
+      <c r="B87" s="8" t="inlineStr">
         <is>
           <t>KR-02 Evidence tracking</t>
         </is>
@@ -1842,7 +1856,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="B89" s="6" t="inlineStr">
+      <c r="B89" s="8" t="inlineStr">
         <is>
           <t>KR-03 Legal-verification case</t>
         </is>
@@ -1872,7 +1886,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="B91" s="6" t="inlineStr">
+      <c r="B91" s="8" t="inlineStr">
         <is>
           <t>KR-04 Document access control</t>
         </is>
@@ -1919,7 +1933,7 @@
       </c>
     </row>
     <row r="94">
-      <c r="B94" s="6" t="inlineStr">
+      <c r="B94" s="8" t="inlineStr">
         <is>
           <t>KR-06 Report versioning</t>
         </is>
@@ -1950,7 +1964,7 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="4" t="inlineStr">
+      <c r="A96" s="7" t="inlineStr">
         <is>
           <t>F – MySecure</t>
         </is>
@@ -1989,7 +2003,7 @@
       </c>
     </row>
     <row r="98">
-      <c r="B98" s="4" t="inlineStr">
+      <c r="B98" s="7" t="inlineStr">
         <is>
           <t>MS-02 Inspection scheduling</t>
         </is>
@@ -2019,7 +2033,7 @@
       </c>
     </row>
     <row r="100">
-      <c r="B100" s="4" t="inlineStr">
+      <c r="B100" s="7" t="inlineStr">
         <is>
           <t>MS-03 Field inspection</t>
         </is>
@@ -2049,7 +2063,7 @@
       </c>
     </row>
     <row r="102">
-      <c r="B102" s="4" t="inlineStr">
+      <c r="B102" s="7" t="inlineStr">
         <is>
           <t>MS-04 Owner report &amp; alerts</t>
         </is>
@@ -2079,7 +2093,7 @@
       </c>
     </row>
     <row r="104">
-      <c r="B104" s="4" t="inlineStr">
+      <c r="B104" s="7" t="inlineStr">
         <is>
           <t>MS-05 Plan history &amp; status</t>
         </is>
@@ -2109,7 +2123,7 @@
       </c>
     </row>
     <row r="106">
-      <c r="B106" s="4" t="inlineStr">
+      <c r="B106" s="7" t="inlineStr">
         <is>
           <t>MS-06 Maintenance/vendor tasks</t>
         </is>
@@ -2139,7 +2153,7 @@
       </c>
     </row>
     <row r="108">
-      <c r="B108" s="4" t="inlineStr">
+      <c r="B108" s="7" t="inlineStr">
         <is>
           <t>MS-07 Area alerts</t>
         </is>
@@ -2170,7 +2184,7 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="6" t="inlineStr">
+      <c r="A110" s="8" t="inlineStr">
         <is>
           <t>G – KONU Buddies / Agent Network</t>
         </is>
@@ -2209,7 +2223,7 @@
       </c>
     </row>
     <row r="112">
-      <c r="B112" s="6" t="inlineStr">
+      <c r="B112" s="8" t="inlineStr">
         <is>
           <t>KB-02 Admin approval</t>
         </is>
@@ -2239,7 +2253,7 @@
       </c>
     </row>
     <row r="114">
-      <c r="B114" s="6" t="inlineStr">
+      <c r="B114" s="8" t="inlineStr">
         <is>
           <t>KB-03 Lead assignment</t>
         </is>
@@ -2269,7 +2283,7 @@
       </c>
     </row>
     <row r="116">
-      <c r="B116" s="6" t="inlineStr">
+      <c r="B116" s="8" t="inlineStr">
         <is>
           <t>KB-04 Mandate/transaction workflow</t>
         </is>
@@ -2299,7 +2313,7 @@
       </c>
     </row>
     <row r="118">
-      <c r="B118" s="6" t="inlineStr">
+      <c r="B118" s="8" t="inlineStr">
         <is>
           <t>KB-05 Quality &amp; feedback</t>
         </is>
@@ -2329,7 +2343,7 @@
       </c>
     </row>
     <row r="120">
-      <c r="B120" s="6" t="inlineStr">
+      <c r="B120" s="8" t="inlineStr">
         <is>
           <t>KB-06 Commission policy</t>
         </is>
@@ -2359,7 +2373,7 @@
       </c>
     </row>
     <row r="122">
-      <c r="B122" s="6" t="inlineStr">
+      <c r="B122" s="8" t="inlineStr">
         <is>
           <t>KB-07 Location-based matching</t>
         </is>
@@ -2390,7 +2404,7 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="4" t="inlineStr">
+      <c r="A124" s="7" t="inlineStr">
         <is>
           <t>H – Developer Services, CRM &amp; Growth Analytics</t>
         </is>
@@ -2429,7 +2443,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="B126" s="4" t="inlineStr">
+      <c r="B126" s="7" t="inlineStr">
         <is>
           <t>DEV-02 Project pages</t>
         </is>
@@ -2459,7 +2473,7 @@
       </c>
     </row>
     <row r="128">
-      <c r="B128" s="4" t="inlineStr">
+      <c r="B128" s="7" t="inlineStr">
         <is>
           <t>DEV-03 Lead capture</t>
         </is>
@@ -2489,7 +2503,7 @@
       </c>
     </row>
     <row r="130">
-      <c r="B130" s="4" t="inlineStr">
+      <c r="B130" s="7" t="inlineStr">
         <is>
           <t>DEV-04 Lead feedback loop</t>
         </is>
@@ -2519,7 +2533,7 @@
       </c>
     </row>
     <row r="132">
-      <c r="B132" s="4" t="inlineStr">
+      <c r="B132" s="7" t="inlineStr">
         <is>
           <t>DEV-05 Funnel analytics</t>
         </is>
@@ -2549,7 +2563,7 @@
       </c>
     </row>
     <row r="134">
-      <c r="B134" s="4" t="inlineStr">
+      <c r="B134" s="7" t="inlineStr">
         <is>
           <t>DEV-06 Commercial model config</t>
         </is>
@@ -2579,7 +2593,7 @@
       </c>
     </row>
     <row r="136">
-      <c r="B136" s="4" t="inlineStr">
+      <c r="B136" s="7" t="inlineStr">
         <is>
           <t>DEV-07 KONU Custom CRM</t>
         </is>
@@ -2622,7 +2636,7 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="6" t="inlineStr">
+      <c r="A139" s="8" t="inlineStr">
         <is>
           <t>I – Admin, Data Ops, Notifications &amp; Platform Controls</t>
         </is>
@@ -2661,7 +2675,7 @@
       </c>
     </row>
     <row r="141">
-      <c r="B141" s="6" t="inlineStr">
+      <c r="B141" s="8" t="inlineStr">
         <is>
           <t>ADM-02 Master data &amp; exceptions</t>
         </is>
@@ -2691,7 +2705,7 @@
       </c>
     </row>
     <row r="143">
-      <c r="B143" s="6" t="inlineStr">
+      <c r="B143" s="8" t="inlineStr">
         <is>
           <t>ADM-03 Notification service</t>
         </is>
@@ -2721,7 +2735,7 @@
       </c>
     </row>
     <row r="145">
-      <c r="B145" s="6" t="inlineStr">
+      <c r="B145" s="8" t="inlineStr">
         <is>
           <t>ADM-04 Pipeline status</t>
         </is>
@@ -2768,7 +2782,7 @@
       </c>
     </row>
     <row r="148">
-      <c r="B148" s="6" t="inlineStr">
+      <c r="B148" s="8" t="inlineStr">
         <is>
           <t>ADM-06 Environment separation</t>
         </is>
@@ -2799,7 +2813,7 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="4" t="inlineStr">
+      <c r="A150" s="7" t="inlineStr">
         <is>
           <t>J – Customer Dashboard</t>
         </is>
@@ -2821,7 +2835,7 @@
       </c>
     </row>
     <row r="151">
-      <c r="B151" s="4" t="inlineStr">
+      <c r="B151" s="7" t="inlineStr">
         <is>
           <t>CD-01 Property activity</t>
         </is>
@@ -2851,7 +2865,7 @@
       </c>
     </row>
     <row r="153">
-      <c r="B153" s="4" t="inlineStr">
+      <c r="B153" s="7" t="inlineStr">
         <is>
           <t>CD-02 Analytics &amp; insights</t>
         </is>
@@ -2881,7 +2895,7 @@
       </c>
     </row>
     <row r="155">
-      <c r="B155" s="4" t="inlineStr">
+      <c r="B155" s="7" t="inlineStr">
         <is>
           <t>CD-03 New-match alerts</t>
         </is>
@@ -2911,7 +2925,7 @@
       </c>
     </row>
     <row r="157">
-      <c r="B157" s="4" t="inlineStr">
+      <c r="B157" s="7" t="inlineStr">
         <is>
           <t>CD-04 Service status</t>
         </is>
@@ -2941,7 +2955,7 @@
       </c>
     </row>
     <row r="159">
-      <c r="B159" s="4" t="inlineStr">
+      <c r="B159" s="7" t="inlineStr">
         <is>
           <t>CD-05 Personalized updates</t>
         </is>
@@ -2987,9 +3001,9 @@
     <mergeCell ref="B102:B103"/>
     <mergeCell ref="A2:A19"/>
     <mergeCell ref="A139:A149"/>
+    <mergeCell ref="B148:B149"/>
+    <mergeCell ref="B73:B74"/>
     <mergeCell ref="B35:B36"/>
-    <mergeCell ref="B73:B74"/>
-    <mergeCell ref="B148:B149"/>
     <mergeCell ref="B145:B146"/>
     <mergeCell ref="B58:B59"/>
     <mergeCell ref="B120:B121"/>
@@ -3023,9 +3037,9 @@
     <mergeCell ref="B54:B55"/>
     <mergeCell ref="B27:B29"/>
     <mergeCell ref="B30:B31"/>
-    <mergeCell ref="B106:B107"/>
     <mergeCell ref="B114:B115"/>
     <mergeCell ref="B136:B138"/>
+    <mergeCell ref="B106:B107"/>
     <mergeCell ref="B79:B80"/>
     <mergeCell ref="B39:B41"/>
     <mergeCell ref="A71:A84"/>
@@ -3054,4 +3068,927 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Sub Task</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>NFR – Platform Requirements</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>NFR-06 Analytics</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Instrument funnel: discovery → lead/service request → fulfilment</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>A – Core Listings, Search &amp; Property Detail</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>CL-07 Duplicate/stale flagging</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Flag duplicate/stale records via admin rules</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>CL-07 Duplicate/stale flagging</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Review without auto-deletion</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>CL-08 Personalized discovery</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Use searches, views, saves, location, budget, configuration, amenities</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Apply consent/privacy controls</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>CL-09 Engagement metrics</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Capture views and saves per listing</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Apply agreed counting rules</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Listing-level analytics</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>B – GIS &amp; Hyperlocal Intelligence</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>GIS-06 Nearby updates</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Detect new properties/developments/infra within approved radius</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>GIS-06 Nearby updates</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Show on dashboard &amp; notification channels</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>C – Kestimate</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>KE-01 Estimate request/view</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Return estimate for supported types/areas</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>KE-01 Estimate request/view</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Insufficient-data state; no fabricated values</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>KE-02 Range/confidence</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Show range/confidence indicator</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>No single unexplained value</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>KE-03 Audit traceability</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Store model version, timestamp, input features</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Apply privacy controls</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>KE-04 Explainability</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Show top value drivers/comparables in plain language</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>KE-05 Data-quality rules</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Define thresholds for missing/stale/outlier inputs</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Fallback behaviour</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="5" t="n"/>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Log exceptions</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>KE-06 Monitoring</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Track errors, latency, coverage, drift/quality</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Segment by geography/property type</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>KE-07 Legal disclaimer</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Show 'informational, not certified valuation' wherever displayed/shared</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>KE-08 GIS-driven refresh</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Use infra/development/connectivity changes as inputs</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n"/>
+      <c r="B26" s="5" t="n"/>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Refresh current estimates &amp; future projections</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>D – Bujji AI Property Assistant</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>AI-01 Grounded answers</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Answer from approved sources &amp; user/property context</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>AI-01 Grounded answers</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>No invented facts</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>AI-02 Uncertainty &amp; escalation</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Indicate insufficient data</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="5" t="n"/>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Bounded response; offer escalation</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>AI-03 Guardrails</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Legal/financial disclaimers</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="5" t="n"/>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Red-team/UAT verification</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>AI-04 Telemetry</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Capture latency, failure, feedback, source IDs</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="5" t="n"/>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Privacy-safe logs; ops can inspect failed/low-rated sessions</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>AI-05 Version control</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Version prompt/model/config</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="5" t="n"/>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Trace responses to deployed version</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>AI-06 Lead routing</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Create lead/service request with consent</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="5" t="n"/>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Include intent summary &amp; property/project ID</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>AI-07 Memory/personalization</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Retain preferences &amp; prior context with consent</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="n"/>
+      <c r="B40" s="5" t="n"/>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Avoid repeated questions</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>G – KONU Buddies / Agent Network</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>KB-07 Location-based matching</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Match by location, service area, proximity, availability</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="n"/>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>KB-07 Location-based matching</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Accept lead; single accountable owner; track status</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>H – Developer Services, CRM &amp; Growth Analytics</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>DEV-05 Funnel analytics</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Document event taxonomy</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="n"/>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>DEV-05 Funnel analytics</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>QA acquisition → engagement → conversion events</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>I – Admin, Data Ops, Notifications &amp; Platform Controls</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>ADM-04 Pipeline status</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Show last success, error, owner</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="n"/>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>ADM-04 Pipeline status</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Identify stale/failed sources</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>J – Customer Dashboard</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>CD-02 Analytics &amp; insights</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Customer-level property analytics</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>CD-02 Analytics &amp; insights</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Insights from activity, preferences, owned properties</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>CD-03 New-match alerts</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Alert on new property matching preferences</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="5" t="n"/>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Card/notification with direct listing link</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>CD-05 Personalized updates</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Notifications &amp; recommendations</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="n"/>
+      <c r="B52" s="5" t="n"/>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Important journey updates</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D52"/>
+  <mergeCells count="23">
+    <mergeCell ref="A3:A9"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="A12:A26"/>
+    <mergeCell ref="B49:B50"/>
+    <mergeCell ref="B33:B34"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A47:A52"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="A27:A40"/>
+    <mergeCell ref="B51:B52"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="B31:B32"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Not Started,In Progress,Done,Blocked"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>